<commit_message>
docs: record the 2026-09-11 chest table agreement and playtest material
Adds the three-chest quality table, the five-question playtest feedback set and
its questionnaire, and refreshes the design workbooks, the localization export
report and the current-goal acceptance pointer to match the shipped tables.

test_gamexxk_localization_catalog.py gains coverage for the chest odds strings
that changed with the loot table.
</commit_message>
<xml_diff>
--- a/docs/design/2026-09-10-project-progress/GameXXK_项目进度与验收总表_2026-09-10.xlsx
+++ b/docs/design/2026-09-10-project-progress/GameXXK_项目进度与验收总表_2026-09-10.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_项目进度" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_完成门槛" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_遗物素材状态" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_共享任务交接" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="01_项目进度" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="02_完成门槛" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="03_遗物素材状态" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="04_共享任务交接" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_项目进度'!$A$4:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01_项目进度'!$A$4:$H$26</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'01_项目进度'!$1:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_完成门槛'!$A$4:$D$31</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'02_完成门槛'!$1:$4</definedName>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -496,7 +496,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11 03:14 +08:00  |  执行中，未完成  |  本次允许根目录 codex/ui-visual-optimization；其他任务结束后统一提交</t>
+          <t>2026-09-11 17:07 +08:00  |  执行中，未完成  |  本次允许根目录 codex/ui-visual-optimization；其他任务结束后统一提交</t>
         </is>
       </c>
     </row>
@@ -1424,8 +1424,50 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>G5P</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>三箱品质概率与宇宙获取路径</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>用户批准三箱一起重列：基点域每列精确10000，珍稀及以上严格1:4:16。讨伐箱采用乙方案：宇宙16bp、天界80bp、登神40bp，是唯一直出顶三档的来源，顶端逐级递减不倒挂；普通箱止于至宝、高级箱止于超凡。九合一采用提案B：每档只前进一档或保持原品质，无跨档跳变，成功率单一平滑递减100/100/100/90/85/80/75/70/60%</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>ResolveLootQuality 改为十档四列（含来源难度）；OpenOneInternal 对普通箱也掷真实随机品质；ToolCombineProbability 改为提案B；设计总表sheet02+sheet04、运行时契约、游戏内 Chest.*.Odds 文本与本地化总表同步</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>冷UBT通过（首次因编辑器占用DLL链接失败，关闭后通过）；GameXXK.Hunt 10/10、Training 50/50、ToolsRedesign 14/14、Localization 21/21；本地化目录测试7/7；10桶609项回归591通过、失败集与改动前完全一致（18项既有红项）</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>实测全队18件宇宙约1.84年（承诺1-2年），其中直出贡献约84%；非地狱讨伐箱路径约11.3年，故地狱讨伐是关键</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>开箱与九合一实机手感复核；用新经济重跑744场矩阵重新判定地狱3-3/3-4定位</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>docs/production/2026-09-11-three-chest-quality-table.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:H25"/>
+  <autoFilter ref="A4:H26"/>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>

</xml_diff>